<commit_message>
Point API tests at the API host and hold runs when the environment drops
The SPA host only serves the app, so /api/* paths under it returned the
app's own HTML 404 instead of reaching the API; API-level tests now read a
separate CBSE_API_BASE_URL. Add environment_health so a dropped network or
an unresponsive API is recognised as infrastructure and the run waits for
the environment instead of burning its retries against a broken one.

Also: M1 group runner and workspace cleanup scripts, Jenkins pipeline docs,
and upload/review page fixes surfaced by the group runs.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/upload_templates/sme_sheet.xlsx
+++ b/data/upload_templates/sme_sheet.xlsx
@@ -681,7 +681,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>acdcc true</t>
+          <t>The learner compares two numbers and judges whether the stated inequality holds.</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -696,11 +696,13 @@
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>xyz</t>
-        </is>
-      </c>
-      <c r="W2" t="n">
-        <v>123</v>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>78 is greater than 45, so the statement 78 &lt; 45 is false.</t>
+        </is>
       </c>
       <c r="X2" t="inlineStr">
         <is>

</xml_diff>